<commit_message>
docs: say why three repositories, and stop asking for a fourth
Asking for 'four repositories' without a reason invites the question, and the answer
was wrong anyway: the fourth is the platform GitOps repository, which either already
exists on the customer side or we bring ourselves. They create three.

The split between code and configuration is not stylistic: the build pushes each
published version into the configuration repository, so sharing one repo would have
that push retrigger the build in a loop. That reason is now stated.

The image repositories were also misstated as something to create -- a playbook
provisions them. What is needed is administrative permission on the registry.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -560,39 +560,43 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Repositorios de código y configuración</t>
+          <t>Repositorio de plataforma: permiso para proponer cambios</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Cuatro repositorios creados, con permiso de escritura para el equipo de implementación.</t>
+          <t>Si ya cuentan con un repositorio de configuración de plataforma, necesitamos poder abrir una solicitud de cambio sobre él. Si no existe, lo aportamos nosotros: no hay que crearlo.</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Se aporta uno nuevo</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Acceso al registro de imágenes</t>
+          <t>Tres repositorios Git vacíos</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Permiso para crear los repositorios de imagen y las cuentas de servicio del proceso de construcción.</t>
+          <t>Uno por cada pieza que evoluciona por separado:
+1) Código del pipeline (Java) — los servicios que descifran y enmascaran.
+2) Código del componente productor (.NET) — la librería que integran sus aplicaciones.
+3) Configuración de despliegue — qué se despliega en cada ambiente.
+Se separa el código de la configuración porque el proceso de construcción escribe en el repositorio de configuración cada versión publicada: en un mismo repositorio, ese cambio volvería a disparar la construcción indefinidamente.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -602,53 +606,74 @@
       </c>
       <c r="E7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Permiso de administración en el registro de imágenes</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>No hay que crear nada a mano: los repositorios de imagen y las cuentas de servicio los crea el equipo de implementación de forma automatizada. Solo se necesita autorización sobre las organizaciones del registro.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Nombre del cluster de Kafka</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Todas las aplicaciones se conectan usando este nombre.</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>demo-kafka</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>Nombre del cluster de Kafka</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>demo-kafka</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
           <t>Nombres de los cuatro tópicos</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>tp.observability.logs.encrypted
 tp.observability.logs.encrypted.dlq
@@ -656,95 +681,74 @@
 tp.observability.logs.masked.dlq</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Nombres de los usuarios de Kafka</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>log-processor
 log-sink
 dummy-data-producer</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Tiempo de retención de los eventos</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Cuánto tiempo se conservan los eventos en Kafka. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>24 horas los tópicos principales
 72 horas las colas de descarte</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Qué campos son datos personales</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>El pipeline enmascara los campos que ustedes declaren como datos personales. Hoy se contemplan el correo, la cédula y el número de tarjeta.</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Correo del cliente
 Cédula (deja visibles 3 dígitos al inicio y 3 al final)
 Número de tarjeta</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Volumen esperado de eventos</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Eventos por segundo y tamaño medio, para dimensionar el cluster correctamente.</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Dimensionado para 2,5 MB por mensaje</t>
-        </is>
-      </c>
       <c r="E14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -753,17 +757,17 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Volumen esperado de eventos</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Eventos por segundo y tamaño medio, para dimensionar el cluster correctamente.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dimensionado para 2,5 MB por mensaje</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
@@ -774,12 +778,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
+          <t>Destino final de los eventos enmascarados</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -795,52 +799,52 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
+          <t>Aplicaciones que enviarán eventos de auditoría</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
           <t>Convención de etiquetas corporativa</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Para etiquetar lo que se despliegue según su estándar (equipo, aplicación, centro de costo).</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Las etiquetas de la configuración base</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>SEGURIDAD Y GOBIERNO</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Llave de cifrado del ambiente</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Es la llave con la que se cifran los eventos. La genera y custodia el cliente; nunca se guarda en el repositorio de código.</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Se genera una para desarrollo</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -848,17 +852,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Gestor de secretos corporativo</t>
+          <t>Llave de cifrado del ambiente</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Cuál se usará para custodiar la llave en los ambientes productivos, y si ya está integrado con OpenShift.</t>
+          <t>Es la llave con la que se cifran los eventos. La genera y custodia el cliente; nunca se guarda en el repositorio de código.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Se genera una para desarrollo</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
@@ -869,20 +873,41 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
+          <t>Gestor de secretos corporativo</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Cuál se usará para custodiar la llave en los ambientes productivos, y si ya está integrado con OpenShift.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
           <t>Política de aprobación de cambios</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr"/>
+      <c r="E22" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: fix the repository ask in the sheet
It asked for four repositories without saying why, and the count was wrong: the
fourth is the platform GitOps repository, which the customer already has or we
bring. Now it asks for three, names each one, and gives the reason they are split --
the build writes each published version into the configuration repository, so a
shared repo would have that push retrigger the build in a loop.

The registry line asked them to create image repositories; a playbook provisions
those, so what is actually needed is permission.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -560,43 +560,43 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="165" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Repositorio de plataforma: permiso para proponer cambios</t>
+          <t>Tres repositorios Git vacíos</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Si ya cuentan con un repositorio de configuración de plataforma, necesitamos poder abrir una solicitud de cambio sobre él. Si no existe, lo aportamos nosotros: no hay que crearlo.</t>
+          <t>1) Código del pipeline (Java)
+2) Código del componente productor (.NET)
+3) Configuración de despliegue
+Van separados porque el proceso de construcción escribe en el repositorio de configuración cada versión publicada: en un mismo repositorio, ese cambio volvería a disparar la construcción en bucle.
+Si además cuentan con un repositorio de plataforma, basta con poder proponerle cambios; si no existe, lo aportamos nosotros.</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Se aporta uno nuevo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="110" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Tres repositorios Git vacíos</t>
+          <t>Permiso de administración en el registro de imágenes</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Uno por cada pieza que evoluciona por separado:
-1) Código del pipeline (Java) — los servicios que descifran y enmascaran.
-2) Código del componente productor (.NET) — la librería que integran sus aplicaciones.
-3) Configuración de despliegue — qué se despliega en cada ambiente.
-Se separa el código de la configuración porque el proceso de construcción escribe en el repositorio de configuración cada versión publicada: en un mismo repositorio, ese cambio volvería a disparar la construcción indefinidamente.</t>
+          <t>Los repositorios de imagen y las cuentas de servicio se crean de forma automatizada; solo hace falta la autorización.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -606,74 +606,53 @@
       </c>
       <c r="E7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="5" t="n">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Permiso de administración en el registro de imágenes</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>No hay que crear nada a mano: los repositorios de imagen y las cuentas de servicio los crea el equipo de implementación de forma automatizada. Solo se necesita autorización sobre las organizaciones del registro.</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Nombre del cluster de Kafka</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>demo-kafka</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Nombre del cluster de Kafka</t>
+          <t>Nombres de los cuatro tópicos</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+          <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>demo-kafka</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Nombres de los cuatro tópicos</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>tp.observability.logs.encrypted
 tp.observability.logs.encrypted.dlq
@@ -681,6 +660,29 @@
 tp.observability.logs.masked.dlq</t>
         </is>
       </c>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Nombres de los usuarios de Kafka</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>log-processor
+log-sink
+dummy-data-producer</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
@@ -689,66 +691,64 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Nombres de los usuarios de Kafka</t>
+          <t>Tiempo de retención de los eventos</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
+          <t>Cuánto tiempo se conservan los eventos en Kafka. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>log-processor
-log-sink
-dummy-data-producer</t>
+          <t>24 horas los tópicos principales
+72 horas las colas de descarte</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Tiempo de retención de los eventos</t>
+          <t>Qué campos son datos personales</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan los eventos en Kafka. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.</t>
+          <t>El pipeline enmascara los campos que ustedes declaren como datos personales. Hoy se contemplan el correo, la cédula y el número de tarjeta.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>24 horas los tópicos principales
-72 horas las colas de descarte</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Qué campos son datos personales</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>El pipeline enmascara los campos que ustedes declaren como datos personales. Hoy se contemplan el correo, la cédula y el número de tarjeta.</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Correo del cliente
 Cédula (deja visibles 3 dígitos al inicio y 3 al final)
 Número de tarjeta</t>
         </is>
       </c>
+      <c r="E13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Volumen esperado de eventos</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Eventos por segundo y tamaño medio, para dimensionar el cluster correctamente.</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Dimensionado para 2,5 MB por mensaje</t>
+        </is>
+      </c>
       <c r="E14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -757,17 +757,17 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Volumen esperado de eventos</t>
+          <t>Destino final de los eventos enmascarados</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo y tamaño medio, para dimensionar el cluster correctamente.</t>
+          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Dimensionado para 2,5 MB por mensaje</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
@@ -778,12 +778,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Aplicaciones que enviarán eventos de auditoría</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -799,52 +799,52 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
+          <t>Convención de etiquetas corporativa</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+          <t>Para etiquetar lo que se despliegue según su estándar (equipo, aplicación, centro de costo).</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Las etiquetas de la configuración base</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="n">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Convención de etiquetas corporativa</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Para etiquetar lo que se despliegue según su estándar (equipo, aplicación, centro de costo).</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Las etiquetas de la configuración base</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Llave de cifrado del ambiente</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Es la llave con la que se cifran los eventos. La genera y custodia el cliente; nunca se guarda en el repositorio de código.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Se genera una para desarrollo</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -852,17 +852,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado del ambiente</t>
+          <t>Gestor de secretos corporativo</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Es la llave con la que se cifran los eventos. La genera y custodia el cliente; nunca se guarda en el repositorio de código.</t>
+          <t>Cuál se usará para custodiar la llave en los ambientes productivos, y si ya está integrado con OpenShift.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Se genera una para desarrollo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
@@ -873,41 +873,20 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Gestor de secretos corporativo</t>
+          <t>Política de aprobación de cambios</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Cuál se usará para custodiar la llave en los ambientes productivos, y si ya está integrado con OpenShift.</t>
+          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Política de aprobación de cambios</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Revisión obligatoria antes de cada promoción</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: name Key Vault as the secret store and put the crypto up for review
The sheet asked which secret manager would be used; it is Azure Key Vault, which
this engagement already runs with External Secrets. The ask is now concrete: which
vault, which secret name, and the Azure identity the cluster reads it with.

Adds a row stating the encryption scheme so the customer's security team can review
it rather than discover it: AES-256-GCM with per-message IV and the topic bound as
authenticated data, 256-bit key derived with HKDF-SHA256, and the delivery service
holding no key at all.

Also sharpens the PII row. Masking covers only the attributes the customer declares,
so anything absent from that list travels unmasked -- that is the claim their
compliance team has to sign off on, and it now says so.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -707,25 +707,26 @@
       </c>
       <c r="E12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="120" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Qué campos son datos personales</t>
+          <t>Catálogo completo de datos personales</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>El pipeline enmascara los campos que ustedes declaren como datos personales. Hoy se contemplan el correo, la cédula y el número de tarjeta.</t>
+          <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
+Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Correo del cliente
 Cédula (deja visibles 3 dígitos al inicio y 3 al final)
-Número de tarjeta</t>
+Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr"/>
@@ -825,68 +826,113 @@
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="195" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado del ambiente</t>
+          <t>Validación del esquema de cifrado por su área de seguridad</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Es la llave con la que se cifran los eventos. La genera y custodia el cliente; nunca se guarda en el repositorio de código.</t>
+          <t>Para su revisión: los eventos se cifran en origen con AES-256-GCM (cifrado autenticado: detecta cualquier manipulación) y cada mensaje queda ligado a su tópico, de modo que copiarlo a otro no se puede descifrar. La llave de 256 bits se deriva con HKDF-SHA256 (RFC 5869 / NIST SP 800-56C) a partir del secreto del Key Vault.
+Los datos personales solo existen en claro dentro del componente que descifra; el servicio que entrega al destino final ni siquiera tiene acceso a la llave.
+Confirmar si su área de seguridad requiere alguna adecuación (por ejemplo, custodia de la llave en HSM).</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Se genera una para desarrollo</t>
+          <t>El esquema descrito</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="120" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Gestor de secretos corporativo</t>
+          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Cuál se usará para custodiar la llave en los ambientes productivos, y si ya está integrado con OpenShift.</t>
+          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
+Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
+          <t>Acceso de OpenShift al Key Vault</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Política de rotación de la llave</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Sin rotación programada en desarrollo</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
           <t>Política de aprobación de cambios</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr"/>
+      <c r="E23" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: ask about network reachability, not about our own crypto
Dropped the row asking the customer to validate the encryption scheme -- we build
that, so it is ours to get right, not theirs to approve.

Added what was genuinely missing: how their .NET applications reach Kafka. Where
they run decides everything else, so that is the first question; then the firewall
opening, name resolution, trusting the cluster certificate and how many client
identities they need. An application that cannot open the connection never gets to
publish an event, and none of that was being asked.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -818,7 +818,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
+          <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
         </is>
       </c>
       <c r="B18" s="4" t="n"/>
@@ -826,113 +826,209 @@
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
     </row>
-    <row r="19" ht="195" customHeight="1">
+    <row r="19" ht="105" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Validación del esquema de cifrado por su área de seguridad</t>
+          <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Para su revisión: los eventos se cifran en origen con AES-256-GCM (cifrado autenticado: detecta cualquier manipulación) y cada mensaje queda ligado a su tópico, de modo que copiarlo a otro no se puede descifrar. La llave de 256 bits se deriva con HKDF-SHA256 (RFC 5869 / NIST SP 800-56C) a partir del secreto del Key Vault.
-Los datos personales solo existen en claro dentro del componente que descifra; el servicio que entrega al destino final ni siquiera tiene acceso a la llave.
-Confirmar si su área de seguridad requiere alguna adecuación (por ejemplo, custodia de la llave en HSM).</t>
+          <t>Determina el camino de red:
+· DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
+· FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>El esquema descrito</t>
+          <t>Se asume que están fuera del cluster</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="120" customHeight="1">
+    <row r="20" ht="75" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>Habilitación de red hacia Kafka</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Resolución de nombres desde las aplicaciones</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="105" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Confianza en el certificado del cluster</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
+Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Autoridad certificadora generada por la plataforma</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Identidad de cada aplicación productora</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Una identidad compartida por ambiente</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
           <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
 Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Un secreto por ambiente en el Key Vault del proyecto</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Acceso de OpenShift al Key Vault</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Política de rotación de la llave</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Sin rotación programada en desarrollo</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Política de aprobación de cambios</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
+      <c r="E28" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: drop the labelling ask, add the topic settings it was hiding
The labelling row asked for a cost-centre convention the manifests never use --
they carry plain technical labels. Asking for something we would not apply is worse
than not asking.

In its place go the settings that were genuinely missing: partition count (it caps
how many instances can process in parallel, and shrinking it later means recreating
the topic), maximum event size, per-application rate limits, and what happens to
messages that fail -- who reviews the dead-letter queue and whether its contents get
reprocessed, archived or dropped. Retention now explains why the dead-letter queues
are kept longer.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="45" customHeight="1">
+    <row r="14" ht="105" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
@@ -742,79 +742,83 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan los eventos en Kafka. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.</t>
+          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
+Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>24 horas los tópicos principales
-72 horas las colas de descarte</t>
+          <t>Tópicos principales: 24 horas
+Colas de descarte: 72 horas</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
     </row>
-    <row r="15" ht="120" customHeight="1">
+    <row r="15" ht="105" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>Qué hacer con los mensajes que fallan</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
+Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>Catálogo completo de datos personales</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
 Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Correo del cliente
 Cédula (deja visibles 3 dígitos al inicio y 3 al final)
 Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Volumen esperado de eventos</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Eventos por segundo y tamaño medio, para dimensionar el cluster correctamente.</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Dimensionado para 2,5 MB por mensaje</t>
-        </is>
-      </c>
       <c r="E16" s="7" t="inlineStr"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="120" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>12</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Volumen esperado y tamaño de los eventos</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
+Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3 particiones por tópico
+Tamaño máximo: 2,5 MB por evento</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr"/>
@@ -825,12 +829,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
+          <t>Destino final de los eventos enmascarados</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -846,183 +850,205 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Convención de etiquetas corporativa</t>
+          <t>Aplicaciones que enviarán eventos de auditoría</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Para etiquetar lo que se despliegue según su estándar (equipo, aplicación, centro de costo).</t>
+          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Las etiquetas de la configuración base</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Límites de consumo por aplicación</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Envío: 2 MB por segundo
+Lectura: 5 MB por segundo</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="105" customHeight="1">
-      <c r="A21" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="105" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Determina el camino de red:
 · DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
 · FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Se asume que están fuera del cluster</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="75" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Habilitación de red hacia Kafka</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="E22" s="7" t="inlineStr"/>
     </row>
-    <row r="23" ht="105" customHeight="1">
+    <row r="23" ht="75" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
+          <t>Habilitación de red hacia Kafka</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="105" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
           <t>Habilitación de red desde el servidor Git hacia el cluster</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
 Sin esta habilitación, la construcción automática no se dispara nunca.</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Resolución de nombres desde las aplicaciones</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="E24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="105" customHeight="1">
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>Resolución de nombres desde las aplicaciones</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26" ht="105" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
           <t>Confianza en el certificado del cluster</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
 Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Autoridad certificadora generada por la plataforma</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Identidad de cada aplicación productora</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Una identidad compartida por ambiente</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="150" customHeight="1">
-      <c r="A28" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="150" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Repositorio interno de paquetes .NET</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Lo que se entrega a sus equipos es un PAQUETE que añaden como dependencia a sus aplicaciones. Hace falta un repositorio interno de paquetes (Azure Artifacts, Nexus, Artifactory u otro) donde publicarlo:
 · Credencial de publicación para el proceso de construcción
@@ -1030,268 +1056,268 @@
 Sin este repositorio, sus aplicaciones no tienen de dónde obtener el componente.</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr"/>
-    </row>
-    <row r="29" ht="120" customHeight="1">
-      <c r="A29" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Versión de .NET de las aplicaciones que lo integrarán</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>El componente está construido sobre .NET 10, la versión con soporte extendido hasta noviembre de 2028. Las aplicaciones que lo integren deben usar esa versión o superior.
 Importante confirmarlo antes de empezar: si sus aplicaciones están en .NET 8 (cuyo soporte termina en noviembre de 2026), hay que acordar si se actualizan o si el componente debe construirse para esa versión.</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>.NET 10</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30" ht="75" customHeight="1">
-      <c r="A30" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31" ht="75" customHeight="1">
+      <c r="A31" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Aprobación de las dependencias del componente</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>SEGURIDAD Y GOBIERNO</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="120" customHeight="1">
-      <c r="A32" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
 Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Un secreto por ambiente en el Key Vault del proyecto</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr"/>
-    </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Acceso de OpenShift al Key Vault</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="E33" s="7" t="inlineStr"/>
     </row>
-    <row r="34" ht="45" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="5" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Acceso de OpenShift al Key Vault</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
+          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Sin rotación programada en desarrollo</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="45" customHeight="1">
       <c r="A35" s="5" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Entrega de credenciales a las aplicaciones externas</t>
+          <t>Política de rotación de la llave</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
+          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Se define durante la implementación</t>
+          <t>Sin rotación programada en desarrollo</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr"/>
     </row>
-    <row r="36" ht="120" customHeight="1">
+    <row r="36" ht="60" customHeight="1">
       <c r="A36" s="5" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
+          <t>Entrega de credenciales a las aplicaciones externas</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Se define durante la implementación</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37" ht="120" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
           <t>Aprobación del catálogo de herramientas de validación</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
 Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>El catálogo propuesto</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr"/>
-    </row>
-    <row r="37" ht="45" customHeight="1">
-      <c r="A37" s="5" t="n">
-        <v>29</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Custodia de la llave de firma de imágenes</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Custodia en el cluster, sin renovación programada</t>
-        </is>
-      </c>
       <c r="E37" s="7" t="inlineStr"/>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="45" customHeight="1">
       <c r="A38" s="5" t="n">
         <v>30</v>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
+          <t>Custodia de la llave de firma de imágenes</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Custodia en el cluster, sin renovación programada</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
           <t>Política de aprobación de cambios</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>ORGANIZACIÓN</t>
         </is>
       </c>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="75" customHeight="1">
-      <c r="A40" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Interlocutor técnico y plazos</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>Un responsable por parte del banco que canalice las autorizaciones anteriores (accesos, cuentas, habilitaciones de red) y una fecha objetivo para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos.</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr"/>
-    </row>
-    <row r="41" ht="45" customHeight="1">
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+    </row>
+    <row r="41" ht="75" customHeight="1">
       <c r="A41" s="5" t="n">
         <v>32</v>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
+          <t>Interlocutor técnico y plazos</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Un responsable por parte del banco que canalice las autorizaciones anteriores (accesos, cuentas, habilitaciones de red) y una fecha objetivo para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos.</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
           <t>Destinatario de las alertas del sistema</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>A dónde deben notificarse las alertas de funcionamiento: correo, herramienta de gestión de incidencias o el canal que utilicen.</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Sin notificación externa en desarrollo</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr"/>
+      <c r="E42" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: frame the credentials as authorisations, drop the alerting ask
The registry and Git rows read like configuration tasks we were handing over. We do
the configuring -- what we cannot do is mint a credential inside the customer's own
organisation. The automation authenticates against their registry and their Git
server, so those two accounts have to come from them. Reworded to say exactly that,
and merged the repository-admin row into the Git one since it is the same account.

Removed the alerting recipient: no alert rules or receivers are configured anywhere
in the platform, so asking who should receive them was asking about something that
does not exist yet. The lone remaining organisational item moved into governance.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -585,18 +585,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="105" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Permiso de administración en el registro de imágenes</t>
+          <t>Cuenta de servicio en el registro de imágenes</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Los repositorios de imagen y las cuentas de servicio se crean de forma automatizada; solo hace falta la autorización.</t>
+          <t>La configuración la hacemos nosotros, pero necesitamos una cuenta con la que hacerlo: los repositorios de imagen y los usuarios de descarga se crean de forma automatizada contra el registro, y esa automatización requiere una credencial con privilegios de administración sobre las organizaciones del proyecto.
+Solo ustedes pueden emitirla si el registro es corporativo.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -606,22 +607,22 @@
       </c>
       <c r="E7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="165" customHeight="1">
+    <row r="8" ht="195" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Cuenta técnica de Git para la automatización</t>
+          <t>Cuenta de servicio en su plataforma Git</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Una cuenta de servicio con:
-· LECTURA de los tres repositorios (para que la herramienta de despliegue los sincronice)
-· ESCRITURA en el repositorio de configuración (el proceso de construcción anota ahí cada versión publicada; es el enlace entre construir y desplegar)
-· Permiso para publicar el resultado de la validación en cada solicitud de cambio
-Sin esta cuenta, lo que se construye nunca llega a desplegarse.</t>
+          <t>Igual que la anterior: la automatización la configuramos nosotros, pero la credencial tiene que salir de su organización. Se necesita una cuenta técnica con:
+· Lectura de los tres repositorios
+· Escritura en el repositorio de configuración — el proceso de construcción anota ahí cada versión publicada, y es lo que enlaza construir con desplegar
+· Permiso de administración sobre los tres repositorios, para dejar configurado el aviso automático que dispara la validación
+Es la única credencial del proyecto que no podemos generar por nuestra cuenta.</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -631,74 +632,53 @@
       </c>
       <c r="E8" s="7" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="5" t="n">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Permiso de administración sobre los tres repositorios</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Para configurar el aviso automático que dispara la validación cuando alguien sube un cambio, y las reglas de protección de la rama principal. Si prefieren configurarlo ustedes, les indicamos los datos exactos.</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Nombre del cluster de Kafka</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>demo-kafka</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Nombre del cluster de Kafka</t>
+          <t>Nombres de los cuatro tópicos</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+          <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>demo-kafka</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Nombres de los cuatro tópicos</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>tp.observability.logs.encrypted
 tp.observability.logs.encrypted.dlq
@@ -706,29 +686,52 @@
 tp.observability.logs.masked.dlq</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Nombres de los usuarios de Kafka</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>log-processor
 log-sink
 dummy-data-producer</t>
         </is>
       </c>
+      <c r="E12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="105" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo de retención de los eventos</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
+Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Tópicos principales: 24 horas
+Colas de descarte: 72 horas</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="105" customHeight="1">
@@ -737,41 +740,42 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Tiempo de retención de los eventos</t>
+          <t>Qué hacer con los mensajes que fallan</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
-Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
+          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
+Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Tópicos principales: 24 horas
-Colas de descarte: 72 horas</t>
+          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
     </row>
-    <row r="15" ht="105" customHeight="1">
+    <row r="15" ht="120" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Qué hacer con los mensajes que fallan</t>
+          <t>Catálogo completo de datos personales</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
-Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
+          <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
+Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
+          <t>Correo del cliente
+Cédula (deja visibles 3 dígitos al inicio y 3 al final)
+Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
@@ -782,43 +786,40 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Catálogo completo de datos personales</t>
+          <t>Volumen esperado y tamaño de los eventos</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
-Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
+          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
+Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Correo del cliente
-Cédula (deja visibles 3 dígitos al inicio y 3 al final)
-Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
+          <t>3 particiones por tópico
+Tamaño máximo: 2,5 MB por evento</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
     </row>
-    <row r="17" ht="120" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>12</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Volumen esperado y tamaño de los eventos</t>
+          <t>Destino final de los eventos enmascarados</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
-Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
+          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>3 particiones por tópico
-Tamaño máximo: 2,5 MB por evento</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr"/>
@@ -829,12 +830,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Aplicaciones que enviarán eventos de auditoría</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -844,95 +845,96 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
+          <t>Límites de consumo por aplicación</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr"/>
-    </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Límites de consumo por aplicación</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Envío: 2 MB por segundo
 Lectura: 5 MB por segundo</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="105" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="105" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Determina el camino de red:
 · DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
 · FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
         </is>
       </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Se asume que están fuera del cluster</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="75" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Habilitación de red hacia Kafka</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+        </is>
+      </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Se asume que están fuera del cluster</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr"/>
     </row>
-    <row r="23" ht="75" customHeight="1">
+    <row r="23" ht="105" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red hacia Kafka</t>
+          <t>Habilitación de red desde el servidor Git hacia el cluster</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+          <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
+Sin esta habilitación, la construcción automática no se dispara nunca.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -942,19 +944,18 @@
       </c>
       <c r="E23" s="7" t="inlineStr"/>
     </row>
-    <row r="24" ht="105" customHeight="1">
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="5" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red desde el servidor Git hacia el cluster</t>
+          <t>Resolución de nombres desde las aplicaciones</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
-Sin esta habilitación, la construcción automática no se dispara nunca.</t>
+          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -964,91 +965,70 @@
       </c>
       <c r="E24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="105" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Resolución de nombres desde las aplicaciones</t>
+          <t>Confianza en el certificado del cluster</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
+          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
+Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Autoridad certificadora generada por la plataforma</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr"/>
     </row>
-    <row r="26" ht="105" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="5" t="n">
         <v>20</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Confianza en el certificado del cluster</t>
+          <t>Identidad de cada aplicación productora</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
-Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
+          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Autoridad certificadora generada por la plataforma</t>
+          <t>Una identidad compartida por ambiente</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr"/>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="5" t="n">
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+    </row>
+    <row r="28" ht="150" customHeight="1">
+      <c r="A28" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Identidad de cada aplicación productora</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Una identidad compartida por ambiente</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-    </row>
-    <row r="29" ht="150" customHeight="1">
-      <c r="A29" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Repositorio interno de paquetes .NET</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Lo que se entrega a sus equipos es un PAQUETE que añaden como dependencia a sus aplicaciones. Hace falta un repositorio interno de paquetes (Azure Artifacts, Nexus, Artifactory u otro) donde publicarlo:
 · Credencial de publicación para el proceso de construcción
@@ -1056,268 +1036,236 @@
 Sin este repositorio, sus aplicaciones no tienen de dónde obtener el componente.</t>
         </is>
       </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Versión de .NET de las aplicaciones que lo integrarán</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>El componente está construido sobre .NET 10, la versión con soporte extendido hasta noviembre de 2028. Las aplicaciones que lo integren deben usar esa versión o superior.
+Importante confirmarlo antes de empezar: si sus aplicaciones están en .NET 8 (cuyo soporte termina en noviembre de 2026), hay que acordar si se actualizan o si el componente debe construirse para esa versión.</t>
+        </is>
+      </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>.NET 10</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr"/>
     </row>
-    <row r="30" ht="120" customHeight="1">
+    <row r="30" ht="75" customHeight="1">
       <c r="A30" s="5" t="n">
         <v>23</v>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Versión de .NET de las aplicaciones que lo integrarán</t>
+          <t>Aprobación de las dependencias del componente</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>El componente está construido sobre .NET 10, la versión con soporte extendido hasta noviembre de 2028. Las aplicaciones que lo integren deben usar esa versión o superior.
-Importante confirmarlo antes de empezar: si sus aplicaciones están en .NET 8 (cuyo soporte termina en noviembre de 2026), hay que acordar si se actualizan o si el componente debe construirse para esa versión.</t>
+          <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>.NET 10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr"/>
     </row>
-    <row r="31" ht="75" customHeight="1">
-      <c r="A31" s="5" t="n">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+    </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Aprobación de las dependencias del componente</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-    </row>
-    <row r="33" ht="120" customHeight="1">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
+Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="60" customHeight="1">
       <c r="A33" s="5" t="n">
         <v>25</v>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
+          <t>Acceso de OpenShift al Key Vault</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
-Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
+          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr"/>
     </row>
-    <row r="34" ht="60" customHeight="1">
+    <row r="34" ht="45" customHeight="1">
       <c r="A34" s="5" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Acceso de OpenShift al Key Vault</t>
+          <t>Política de rotación de la llave</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
+          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sin rotación programada en desarrollo</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr"/>
     </row>
-    <row r="35" ht="45" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="5" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Entrega de credenciales a las aplicaciones externas</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
+          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Sin rotación programada en desarrollo</t>
+          <t>Se define durante la implementación</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr"/>
     </row>
-    <row r="36" ht="60" customHeight="1">
+    <row r="36" ht="120" customHeight="1">
       <c r="A36" s="5" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Entrega de credenciales a las aplicaciones externas</t>
+          <t>Aprobación del catálogo de herramientas de validación</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
+          <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
+Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Se define durante la implementación</t>
+          <t>El catálogo propuesto</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr"/>
     </row>
-    <row r="37" ht="120" customHeight="1">
+    <row r="37" ht="45" customHeight="1">
       <c r="A37" s="5" t="n">
         <v>29</v>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Aprobación del catálogo de herramientas de validación</t>
+          <t>Custodia de la llave de firma de imágenes</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
-Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
+          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>El catálogo propuesto</t>
+          <t>Custodia en el cluster, sin renovación programada</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr"/>
     </row>
-    <row r="38" ht="45" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="5" t="n">
         <v>30</v>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Custodia de la llave de firma de imágenes</t>
+          <t>Política de aprobación de cambios</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
+          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Custodia en el cluster, sin renovación programada</t>
+          <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr"/>
     </row>
-    <row r="39" ht="30" customHeight="1">
+    <row r="39" ht="60" customHeight="1">
       <c r="A39" s="5" t="n">
         <v>31</v>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Política de aprobación de cambios</t>
+          <t>Interlocutor técnico y fecha objetivo</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
+          <t>Un responsable por parte del banco que canalice las autorizaciones de este documento y una fecha para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos al inicio.</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Revisión obligatoria antes de cada promoción</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr"/>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>ORGANIZACIÓN</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="75" customHeight="1">
-      <c r="A41" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>Interlocutor técnico y plazos</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Un responsable por parte del banco que canalice las autorizaciones anteriores (accesos, cuentas, habilitaciones de red) y una fecha objetivo para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos.</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr"/>
-    </row>
-    <row r="42" ht="45" customHeight="1">
-      <c r="A42" s="5" t="n">
-        <v>33</v>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Destinatario de las alertas del sistema</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>A dónde deben notificarse las alertas de funcionamiento: correo, herramienta de gestión de incidencias o el canal que utilicen.</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Sin notificación externa en desarrollo</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: fold the credential ask into the repository row
Two separate rows asked for service accounts on the registry and on Git, which read
as work being handed to the customer. The registry one goes entirely -- that is ours
to set up. What is left of the Git one is a clause inside the repository row, where
it belongs: we configure the automation, its credential has to come from their
organisation.

Access asks are down to two: the cluster and the repositories.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -560,13 +560,13 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="165" customHeight="1">
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Tres repositorios Git vacíos</t>
+          <t>Tres repositorios Git y acceso de administración</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -574,111 +574,64 @@
           <t>1) Código del pipeline (Java)
 2) Código del componente productor (.NET)
 3) Configuración de despliegue
-Van separados porque el proceso de construcción escribe en el repositorio de configuración cada versión publicada: en un mismo repositorio, ese cambio volvería a disparar la construcción en bucle.
-Si además cuentan con un repositorio de plataforma, basta con poder proponerle cambios; si no existe, lo aportamos nosotros.</t>
+Separados porque la construcción escribe en el de configuración cada versión publicada: juntos, ese cambio dispararía la construcción en bucle.
+La automatización la configuramos nosotros, pero su credencial debe emitirse desde su organización.</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Si tienen repositorio de plataforma, basta con poder proponerle cambios; si no, lo aportamos</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="105" customHeight="1">
-      <c r="A7" s="5" t="n">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Cuenta de servicio en el registro de imágenes</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>La configuración la hacemos nosotros, pero necesitamos una cuenta con la que hacerlo: los repositorios de imagen y los usuarios de descarga se crean de forma automatizada contra el registro, y esa automatización requiere una credencial con privilegios de administración sobre las organizaciones del proyecto.
-Solo ustedes pueden emitirla si el registro es corporativo.</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8" ht="195" customHeight="1">
-      <c r="A8" s="5" t="n">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Nombre del cluster de Kafka</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Todas las aplicaciones se conectan usando este nombre.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>demo-kafka</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Cuenta de servicio en su plataforma Git</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Igual que la anterior: la automatización la configuramos nosotros, pero la credencial tiene que salir de su organización. Se necesita una cuenta técnica con:
-· Lectura de los tres repositorios
-· Escritura en el repositorio de configuración — el proceso de construcción anota ahí cada versión publicada, y es lo que enlaza construir con desplegar
-· Permiso de administración sobre los tres repositorios, para dejar configurado el aviso automático que dispara la validación
-Es la única credencial del proyecto que no podemos generar por nuestra cuenta.</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>DEFINICIONES DE NEGOCIO   ·   cambiarlas después obliga a modificar todas las aplicaciones ya integradas</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Nombre del cluster de Kafka</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Todas las aplicaciones se conectan usando este nombre.</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>demo-kafka</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Nombres de los cuatro tópicos</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>tp.observability.logs.encrypted
 tp.observability.logs.encrypted.dlq
@@ -686,197 +639,241 @@
 tp.observability.logs.masked.dlq</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Nombres de los usuarios de Kafka</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>log-processor
 log-sink
 dummy-data-producer</t>
         </is>
       </c>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo de retención de los eventos</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
+Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Tópicos principales: 24 horas
+Colas de descarte: 72 horas</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Qué hacer con los mensajes que fallan</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
+Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="105" customHeight="1">
+    <row r="13" ht="120" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Tiempo de retención de los eventos</t>
+          <t>Catálogo completo de datos personales</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
-Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Tópicos principales: 24 horas
-Colas de descarte: 72 horas</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14" ht="105" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Qué hacer con los mensajes que fallan</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
-Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="120" customHeight="1">
-      <c r="A15" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Catálogo completo de datos personales</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
 Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Correo del cliente
 Cédula (deja visibles 3 dígitos al inicio y 3 al final)
 Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
         </is>
       </c>
+      <c r="E13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Volumen esperado y tamaño de los eventos</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
+Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>3 particiones por tópico
+Tamaño máximo: 2,5 MB por evento</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Destino final de los eventos enmascarados</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="inlineStr"/>
     </row>
-    <row r="16" ht="120" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="n">
         <v>11</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Volumen esperado y tamaño de los eventos</t>
+          <t>Aplicaciones que enviarán eventos de auditoría</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
-Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
+          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>3 particiones por tópico
-Tamaño máximo: 2,5 MB por evento</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>12</v>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Límites de consumo por aplicación</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Límites de consumo por aplicación</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Envío: 2 MB por segundo
 Lectura: 5 MB por segundo</t>
         </is>
       </c>
+      <c r="E17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="105" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Determina el camino de red:
+· DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
+· FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Se asume que están fuera del cluster</t>
+        </is>
+      </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
+    <row r="20" ht="75" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Habilitación de red hacia Kafka</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="105" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -884,35 +881,34 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
+          <t>Habilitación de red desde el servidor Git hacia el cluster</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Determina el camino de red:
-· DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
-· FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
+          <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
+Sin esta habilitación, la construcción automática no se dispara nunca.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Se asume que están fuera del cluster</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr"/>
     </row>
-    <row r="22" ht="75" customHeight="1">
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="5" t="n">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red hacia Kafka</t>
+          <t>Resolución de nombres desde las aplicaciones</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -928,107 +924,64 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red desde el servidor Git hacia el cluster</t>
+          <t>Confianza en el certificado del cluster</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
-Sin esta habilitación, la construcción automática no se dispara nunca.</t>
+          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
+Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Autoridad certificadora generada por la plataforma</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr"/>
     </row>
-    <row r="24" ht="45" customHeight="1">
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="5" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Resolución de nombres desde las aplicaciones</t>
+          <t>Identidad de cada aplicación productora</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
+          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Una identidad compartida por ambiente</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="105" customHeight="1">
-      <c r="A25" s="5" t="n">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+    </row>
+    <row r="26" ht="150" customHeight="1">
+      <c r="A26" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Confianza en el certificado del cluster</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
-Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Autoridad certificadora generada por la plataforma</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="5" t="n">
-        <v>20</v>
-      </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Identidad de cada aplicación productora</t>
+          <t>Repositorio interno de paquetes .NET</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Una identidad compartida por ambiente</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="150" customHeight="1">
-      <c r="A28" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Repositorio interno de paquetes .NET</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Lo que se entrega a sus equipos es un PAQUETE que añaden como dependencia a sus aplicaciones. Hace falta un repositorio interno de paquetes (Azure Artifacts, Nexus, Artifactory u otro) donde publicarlo:
 · Credencial de publicación para el proceso de construcción
@@ -1036,85 +989,127 @@
 Sin este repositorio, sus aplicaciones no tienen de dónde obtener el componente.</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr"/>
-    </row>
-    <row r="29" ht="120" customHeight="1">
-      <c r="A29" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Versión de .NET de las aplicaciones que lo integrarán</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>El componente está construido sobre .NET 10, la versión con soporte extendido hasta noviembre de 2028. Las aplicaciones que lo integren deben usar esa versión o superior.
 Importante confirmarlo antes de empezar: si sus aplicaciones están en .NET 8 (cuyo soporte termina en noviembre de 2026), hay que acordar si se actualizan o si el componente debe construirse para esa versión.</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>.NET 10</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30" ht="75" customHeight="1">
+      <c r="E27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28" ht="75" customHeight="1">
+      <c r="A28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Aprobación de las dependencias del componente</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+    </row>
+    <row r="30" ht="120" customHeight="1">
       <c r="A30" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
+Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Aprobación de las dependencias del componente</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Acceso de OpenShift al Key Vault</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="120" customHeight="1">
+      <c r="E31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="45" customHeight="1">
       <c r="A32" s="5" t="n">
         <v>24</v>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
+          <t>Política de rotación de la llave</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
-Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
+          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
+          <t>Sin rotación programada en desarrollo</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr"/>
@@ -1125,147 +1120,105 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Acceso de OpenShift al Key Vault</t>
+          <t>Entrega de credenciales a las aplicaciones externas</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
+          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Se define durante la implementación</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr"/>
     </row>
-    <row r="34" ht="45" customHeight="1">
+    <row r="34" ht="120" customHeight="1">
       <c r="A34" s="5" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Aprobación del catálogo de herramientas de validación</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
+          <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
+Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Sin rotación programada en desarrollo</t>
+          <t>El catálogo propuesto</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="45" customHeight="1">
       <c r="A35" s="5" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Entrega de credenciales a las aplicaciones externas</t>
+          <t>Custodia de la llave de firma de imágenes</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
+          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Se define durante la implementación</t>
+          <t>Custodia en el cluster, sin renovación programada</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr"/>
     </row>
-    <row r="36" ht="120" customHeight="1">
+    <row r="36" ht="30" customHeight="1">
       <c r="A36" s="5" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Aprobación del catálogo de herramientas de validación</t>
+          <t>Política de aprobación de cambios</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
-Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
+          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>El catálogo propuesto</t>
+          <t>Revisión obligatoria antes de cada promoción</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr"/>
     </row>
-    <row r="37" ht="45" customHeight="1">
+    <row r="37" ht="60" customHeight="1">
       <c r="A37" s="5" t="n">
         <v>29</v>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Custodia de la llave de firma de imágenes</t>
+          <t>Interlocutor técnico y fecha objetivo</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
+          <t>Un responsable por parte del banco que canalice las autorizaciones de este documento y una fecha para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos al inicio.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Custodia en el cluster, sin renovación programada</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Política de aprobación de cambios</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Revisión obligatoria antes de cada promoción</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr"/>
-    </row>
-    <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>Interlocutor técnico y fecha objetivo</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Un responsable por parte del banco que canalice las autorizaciones de este documento y una fecha para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos al inicio.</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: shorten every explanation and drop what is theirs to run
The 'Para qué' column had grown into paragraphs justifying each ask. One or two
sentences carry the same weight in a document meant to be read once and answered.

Also removed five rows that told the bank how to organise itself rather than asking
for something we need: who reviews the dead-letter queue, who approves dependencies
and CI tooling, who signs off promotions, and naming a counterpart. All internal
management. What we need is the data and the access; how they govern it is theirs.

Down to 24 asks.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>ACCESOS   ·   lo que necesitamos para poder trabajar</t>
+          <t>ACCESOS</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -539,7 +539,7 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
@@ -550,7 +550,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Credenciales con permisos de administrador para el equipo de implementación. El resto de condiciones del cluster (almacenamiento, salida a los catálogos, capacidad) las verificamos nosotros al instalar.</t>
+          <t>Credenciales de administrador para el equipo de implementación. Las condiciones técnicas del cluster las verificamos nosotros.</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="150" customHeight="1">
+    <row r="6" ht="75" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
@@ -571,10 +571,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>1) Código del pipeline (Java)
-2) Código del componente productor (.NET)
-3) Configuración de despliegue
-Separados porque la construcción escribe en el de configuración cada versión publicada: juntos, ese cambio dispararía la construcción en bucle.
+          <t>Uno para el código del pipeline (Java), otro para el componente productor (.NET) y otro para la configuración de despliegue.
 La automatización la configuramos nosotros, pero su credencial debe emitirse desde su organización.</t>
         </is>
       </c>
@@ -628,7 +625,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Se necesitan: uno para los eventos cifrados que envían las aplicaciones, otro para los eventos ya enmascarados, y una cola de descarte para cada uno (donde van los mensajes que no se pudieron procesar).</t>
+          <t>Dos para el flujo (eventos cifrados y eventos enmascarados) y una cola de descarte para cada uno.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -652,7 +649,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Una identidad por servicio, con permisos mínimos. Aparecen en los registros de acceso y en las métricas.</t>
+          <t>Una identidad por servicio, con permisos mínimos.</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -664,7 +661,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr"/>
     </row>
-    <row r="11" ht="105" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
@@ -675,8 +672,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan los eventos antes de eliminarse. Es una decisión de cumplimiento: define hasta cuándo se puede auditar o reprocesar un evento.
-Las colas de descarte se conservan más tiempo a propósito: son los mensajes que fallaron y hay que poder analizarlos antes de que desaparezcan.</t>
+          <t>Cuánto tiempo se conservan antes de eliminarse. Es una decisión de cumplimiento.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -687,71 +683,68 @@
       </c>
       <c r="E11" s="7" t="inlineStr"/>
     </row>
-    <row r="12" ht="105" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="5" t="n">
         <v>7</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Qué hacer con los mensajes que fallan</t>
+          <t>Catálogo completo de datos personales</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Un evento que no se puede procesar (llega dañado, o cifrado con una llave que ya no está vigente) se aparta en una cola de descarte en lugar de detener el flujo o perderse.
-Confirmar quién revisa esa cola, con qué frecuencia y qué se hace con lo que contiene: reprocesar, archivar o descartar tras el plazo de retención.</t>
+          <t>Se enmascaran ÚNICAMENTE los campos que ustedes declaren: lo que no esté en la lista viaja sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Se aparta y se conserva 72 horas; sin proceso de revisión definido</t>
+          <t>Correo del cliente
+Cédula (deja visibles 3 dígitos al inicio y 3 al final)
+Número de tarjeta (deja los últimos 4)</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="120" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Catálogo completo de datos personales</t>
+          <t>Volumen y tamaño de los eventos</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>El pipeline enmascara ÚNICAMENTE los campos que ustedes declaren. Hoy se contemplan tres: correo, cédula y número de tarjeta.
-Es el punto más sensible del documento: cualquier dato personal que no esté en esta lista (nombres, números de cuenta, teléfonos, direcciones) viajaría sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
+          <t>Eventos por segundo, tamaño medio y máximo. De aquí sale el número de particiones, que después no se puede reducir.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Correo del cliente
-Cédula (deja visibles 3 dígitos al inicio y 3 al final)
-Número de tarjeta (deja los últimos 4, según PCI DSS)</t>
+          <t>3 particiones por tópico
+Tamaño máximo: 2,5 MB por evento</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="120" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Volumen esperado y tamaño de los eventos</t>
+          <t>Destino final de los eventos enmascarados</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo, tamaño medio y tamaño máximo previsto. De aquí sale el número de particiones de cada tópico, que es lo que determina cuántas instancias pueden procesar en paralelo: ampliarlo después es posible, pero reducirlo obliga a recrear el tópico.
-Un evento por encima del tamaño máximo se rechaza en el envío, así que conviene fijarlo con margen.</t>
+          <t>A dónde se entregan una vez procesados: sistema destino, punto de conexión y credenciales.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>3 particiones por tópico
-Tamaño máximo: 2,5 MB por evento</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
@@ -762,12 +755,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>Aplicaciones que enviarán eventos</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>A dónde deben entregarse los eventos una vez descifrados y enmascarados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Cuáles integrarán el componente productor, para planificar la integración.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -783,89 +776,87 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos de auditoría</t>
+          <t>Límites de consumo por aplicación</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Qué aplicaciones integrarán el componente productor y en qué lenguaje están, para planificar la integración.</t>
+          <t>Límite de velocidad por aplicación, para que un fallo en una no afecte a las demás.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Límites de consumo por aplicación</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación tiene un límite de velocidad de envío y de lectura, para que un fallo en una de ellas no sature el servicio para las demás. Confirmar si los valores propuestos son adecuados al volumen real.</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Envío: 2 MB por segundo
 Lectura: 5 MB por segundo</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>CONECTIVIDAD DE LAS APLICACIONES   ·   cómo llegan sus aplicaciones .NET hasta Kafka</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="105" customHeight="1">
+      <c r="E16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>CONECTIVIDAD DE LAS APLICACIONES</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Dónde se ejecutan las aplicaciones</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Si están dentro del cluster no hay que abrir nada; si están fuera, hay que habilitar el tránsito hasta él.</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Se asume que están fuera del cluster</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Dónde se ejecutan las aplicaciones que enviarán eventos</t>
+          <t>Habilitación de red hacia Kafka</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Determina el camino de red:
-· DENTRO del mismo cluster — se conectan por la red interna. No hace falta abrir nada.
-· FUERA del cluster (otro cluster, servidores propios o máquinas virtuales) — se conectan a través de una dirección publicada, y hay que habilitar el tránsito hasta ella.</t>
+          <t>Solo si están fuera: permitir el tránsito desde sus redes hacia Kafka por HTTPS (443). Indicar desde qué redes se originará.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Se asume que están fuera del cluster</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="75" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red hacia Kafka</t>
+          <t>Habilitación de red desde el servidor Git</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Solo si las aplicaciones están fuera del cluster: permitir el tránsito desde sus redes hacia la dirección publicada de Kafka, por HTTPS (puerto 443). Necesitamos saber desde qué redes o segmentos se originará el tráfico para solicitar la habilitación.</t>
+          <t>El servidor Git avisa al cluster cuando alguien sube un cambio. Sin este permiso, la construcción no se dispara.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -875,19 +866,18 @@
       </c>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="105" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red desde el servidor Git hacia el cluster</t>
+          <t>Resolución de nombres</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>En sentido contrario al anterior: cuando alguien sube un cambio, el servidor Git avisa al cluster para que arranque la validación. Requiere permitir ese tránsito, por HTTPS (443), desde el servidor Git hacia la dirección publicada del cluster.
-Sin esta habilitación, la construcción automática no se dispara nunca.</t>
+          <t>Las aplicaciones se conectan por nombre. Confirmar que sus servidores resuelven el dominio del cluster.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -903,322 +893,210 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Resolución de nombres desde las aplicaciones</t>
+          <t>Confianza en el certificado del cluster</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones se conectan por nombre, no por dirección IP. Confirmar que sus servidores resuelven el dominio del cluster; si usan un DNS interno, puede requerir una entrada adicional.</t>
+          <t>Las aplicaciones deben confiar en el certificado que presenta Kafka. Indicar si prefieren emitirlo con su autoridad corporativa.</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Autoridad generada por la plataforma</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr"/>
     </row>
-    <row r="23" ht="105" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Confianza en el certificado del cluster</t>
+          <t>Identidad de cada aplicación productora</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>La conexión va cifrada y las aplicaciones deben confiar en el certificado que presenta Kafka. Se entrega el certificado de la autoridad correspondiente para incorporarlo al almacén de confianza de cada aplicación.
-Indicar si prefieren que el certificado lo emita su autoridad certificadora corporativa.</t>
+          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta y cómo se les entrega.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Autoridad certificadora generada por la plataforma</t>
+          <t>Una identidad compartida por ambiente</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr"/>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="5" t="n">
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Identidad de cada aplicación productora</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Cada aplicación se autentica con su propio certificado de cliente, que emitimos nosotros. Se necesita saber cuántas identidades distintas hacen falta y cómo se les hará llegar su credencial.</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Una identidad compartida por ambiente</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES   ·   cómo lo incorporan sus equipos de desarrollo</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-    </row>
-    <row r="26" ht="150" customHeight="1">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Repositorio interno de paquetes .NET</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Sus equipos incorporan el componente como dependencia: hace falta un repositorio interno donde publicarlo.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="n">
         <v>19</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Repositorio interno de paquetes .NET</t>
+          <t>Versión de .NET de las aplicaciones</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Lo que se entrega a sus equipos es un PAQUETE que añaden como dependencia a sus aplicaciones. Hace falta un repositorio interno de paquetes (Azure Artifacts, Nexus, Artifactory u otro) donde publicarlo:
-· Credencial de publicación para el proceso de construcción
-· Acceso de lectura para sus equipos de desarrollo
-Sin este repositorio, sus aplicaciones no tienen de dónde obtener el componente.</t>
+          <t>El componente está construido sobre .NET 10. Confirmar la versión de las aplicaciones que lo integrarán.</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
+          <t>.NET 10</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Llave de cifrado en Azure Key Vault</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Se deposita en el Key Vault y desde ahí se sincroniza al cluster. Confirmar cuál usar y el nombre del secreto.</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Un secreto por ambiente</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Acceso de OpenShift al Key Vault</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Una identidad de Azure con permiso de lectura sobre el Key Vault.</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="120" customHeight="1">
-      <c r="A27" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Versión de .NET de las aplicaciones que lo integrarán</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>El componente está construido sobre .NET 10, la versión con soporte extendido hasta noviembre de 2028. Las aplicaciones que lo integren deben usar esa versión o superior.
-Importante confirmarlo antes de empezar: si sus aplicaciones están en .NET 8 (cuyo soporte termina en noviembre de 2026), hay que acordar si se actualizan o si el componente debe construirse para esa versión.</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>.NET 10</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="75" customHeight="1">
-      <c r="A28" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Aprobación de las dependencias del componente</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>El paquete incorpora bibliotecas de terceros de uso extendido para conectarse a Kafka y para el formato de los eventos. Si su organización exige revisión previa de dependencias, conviene iniciarla al comienzo del proyecto para no bloquear la integración al final.</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="120" customHeight="1">
+      <c r="E29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="5" t="n">
         <v>22</v>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado del ambiente, en Azure Key Vault</t>
+          <t>Política de rotación de la llave</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Es la llave con la que se cifran los eventos. Se deposita en el Key Vault corporativo y desde ahí se sincroniza al cluster de forma automática: no se guarda en el repositorio de código ni se entrega por otro medio. Se necesita una llave DISTINTA por ambiente.
-Confirmar el Key Vault a utilizar para desarrollo y el nombre del secreto según su estándar de nomenclatura.</t>
+          <t>Cada cuánto debe rotarse. La rotación no pierde los eventos ya publicados.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Un secreto por ambiente en el Key Vault del proyecto</t>
+          <t>Sin rotación programada en desarrollo</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr"/>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31" ht="30" customHeight="1">
       <c r="A31" s="5" t="n">
         <v>23</v>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Acceso de OpenShift al Key Vault</t>
+          <t>Entrega de credenciales a aplicaciones externas</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>El cluster lee los secretos mediante una identidad de Azure con permiso de lectura sobre el Key Vault. Se necesita esa identidad (o autorización para crearla) y confirmar que hay conectividad desde el cluster.</t>
+          <t>Solo si hay aplicaciones fuera del cluster: cómo se les hace llegar su certificado y la llave.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Se define durante la implementación</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr"/>
     </row>
-    <row r="32" ht="45" customHeight="1">
+    <row r="32" ht="30" customHeight="1">
       <c r="A32" s="5" t="n">
         <v>24</v>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Custodia de la llave de firma</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse la llave de cifrado. El sistema admite rotación sin pérdida de datos: durante la transición convive con la llave anterior para poder descifrar lo ya publicado.</t>
+          <t>Las imágenes se firman para verificar su origen. Definir quién custodia la llave.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Sin rotación programada en desarrollo</t>
+          <t>Custodia en el cluster</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr"/>
-    </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Entrega de credenciales a las aplicaciones externas</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Solo si las aplicaciones productoras se ejecutan fuera del cluster: cada una necesita su certificado de cliente y la llave de cifrado en su propio servidor. Acordar cómo se les hace llegar ese material y cómo se renueva cuando caduque o rote.</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Se define durante la implementación</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr"/>
-    </row>
-    <row r="34" ht="120" customHeight="1">
-      <c r="A34" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Aprobación del catálogo de herramientas de validación</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>El proceso de construcción usa herramientas de análisis de código, inventario de componentes y detección de credenciales que son de código abierto y no forman parte del catálogo de Red Hat. Se publican en su propio registro, nunca se descargan de internet en cada ejecución.
-Si su área de seguridad debe aprobarlas, conviene iniciarlo al comienzo.</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>El catálogo propuesto</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr"/>
-    </row>
-    <row r="35" ht="45" customHeight="1">
-      <c r="A35" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>Custodia de la llave de firma de imágenes</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Cada imagen se firma para poder verificar su origen antes de desplegarla. La llave la generamos nosotros; definir quién la custodia y con qué periodicidad se renueva.</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Custodia en el cluster, sin renovación programada</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Política de aprobación de cambios</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Quién aprueba el paso de una versión a los ambientes superiores.</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Revisión obligatoria antes de cada promoción</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr"/>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="5" t="n">
-        <v>29</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Interlocutor técnico y fecha objetivo</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Un responsable por parte del banco que canalice las autorizaciones de este documento y una fecha para tenerlas. Varias dependen de áreas distintas —redes, seguridad, desarrollo— y son la causa más frecuente de retrasos al inicio.</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
fix(kafka): expose the broker through the load balancer, not a Route
MetalLB is deployed with its address pools, but Kafka never used it: the external
listener was still type route. A Route routes by hostname over HTTP, and the Kafka
protocol is binary over TCP -- an external client would not have connected at all.

It now takes an address from the pool. Kafka needs one per broker plus a bootstrap
address, so the prerequisites sheet asks for the range and the port: the pool in Git
carries an example range that has to be replaced with the customer's real segment,
and the firewall row now points at those addresses instead of 443.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -824,60 +824,60 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red hacia Kafka</t>
+          <t>Direcciones IP para exponer Kafka</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Solo si están fuera: permitir el tránsito desde sus redes hacia Kafka por HTTPS (443). Indicar desde qué redes se originará.</t>
+          <t>La exposición se hace con un balanceador que toma direcciones de un rango del segmento de red del cluster. Se necesita una dirección por broker más una de entrada: 2 para desarrollo.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rango a definir con su equipo de redes</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red desde el servidor Git</t>
+          <t>Puerto de conexión a Kafka</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>El servidor Git avisa al cluster cuando alguien sube un cambio. Sin este permiso, la construcción no se dispara.</t>
+          <t>El puerto por el que las aplicaciones se conectan al balanceador. Confirmar si el propuesto es válido según su normativa de red.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9094</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Resolución de nombres</t>
+          <t>Habilitación de red hacia Kafka</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones se conectan por nombre. Confirmar que sus servidores resuelven el dominio del cluster.</t>
+          <t>Solo si están fuera: permitir el tránsito desde sus redes hacia esas direcciones y ese puerto. Indicar desde qué redes se originará.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -887,23 +887,23 @@
       </c>
       <c r="E21" s="7" t="inlineStr"/>
     </row>
-    <row r="22" ht="45" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="n">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Confianza en el certificado del cluster</t>
+          <t>Habilitación de red desde el servidor Git</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones deben confiar en el certificado que presenta Kafka. Indicar si prefieren emitirlo con su autoridad corporativa.</t>
+          <t>El servidor Git avisa al cluster cuando alguien sube un cambio. Sin este permiso, la construcción no se dispara.</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Autoridad generada por la plataforma</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr"/>
@@ -914,126 +914,126 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Identidad de cada aplicación productora</t>
+          <t>Resolución de nombres</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta y cómo se les entrega.</t>
+          <t>Las aplicaciones se conectan por nombre. Confirmar que sus servidores resuelven el dominio del cluster.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Una identidad compartida por ambiente</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr"/>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Confianza en el certificado del cluster</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Las aplicaciones deben confiar en el certificado que presenta Kafka. Indicar si prefieren emitirlo con su autoridad corporativa.</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Autoridad generada por la plataforma</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>Identidad de cada aplicación productora</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta y cómo se les entrega.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Una identidad compartida por ambiente</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>ENTREGA DEL COMPONENTE A SUS APLICACIONES</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
           <t>Repositorio interno de paquetes .NET</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Sus equipos incorporan el componente como dependencia: hace falta un repositorio interno donde publicarlo.</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Versión de .NET de las aplicaciones</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>El componente está construido sobre .NET 10. Confirmar la versión de las aplicaciones que lo integrarán.</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>.NET 10</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>SEGURIDAD Y GOBIERNO</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
+      <c r="E27" s="7" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado en Azure Key Vault</t>
+          <t>Versión de .NET de las aplicaciones</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Se deposita en el Key Vault y desde ahí se sincroniza al cluster. Confirmar cuál usar y el nombre del secreto.</t>
+          <t>El componente está construido sobre .NET 10. Confirmar la versión de las aplicaciones que lo integrarán.</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Un secreto por ambiente</t>
+          <t>.NET 10</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Acceso de OpenShift al Key Vault</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Una identidad de Azure con permiso de lectura sobre el Key Vault.</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr"/>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>SEGURIDAD Y GOBIERNO</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="5" t="n">
@@ -1041,17 +1041,17 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Llave de cifrado en Azure Key Vault</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse. La rotación no pierde los eventos ya publicados.</t>
+          <t>Se deposita en el Key Vault y desde ahí se sincroniza al cluster. Confirmar cuál usar y el nombre del secreto.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Sin rotación programada en desarrollo</t>
+          <t>Un secreto por ambiente</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr"/>
@@ -1062,17 +1062,17 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Entrega de credenciales a aplicaciones externas</t>
+          <t>Acceso de OpenShift al Key Vault</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Solo si hay aplicaciones fuera del cluster: cómo se les hace llegar su certificado y la llave.</t>
+          <t>Una identidad de Azure con permiso de lectura sobre el Key Vault.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Se define durante la implementación</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr"/>
@@ -1083,20 +1083,62 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>Política de rotación de la llave</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Cada cuánto debe rotarse. La rotación no pierde los eventos ya publicados.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Sin rotación programada en desarrollo</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Entrega de credenciales a aplicaciones externas</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Solo si hay aplicaciones fuera del cluster: cómo se les hace llegar su certificado y la llave.</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Se define durante la implementación</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
           <t>Custodia de la llave de firma</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Las imágenes se firman para verificar su origen. Definir quién custodia la llave.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Custodia en el cluster</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr"/>
+      <c r="E34" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs: let the customer set the port, and say it is a range
The port row proposed 9094 as though it were fixed. It is theirs to choose under
their own network policy, and it is not a single port: the load balancer takes one
per broker on top of the bootstrap one, consecutively. Agreeing on 9094 means 9094
and 9095 get used in development.

Same for the addresses -- they have to be free and reserved, or another team takes
them and the service stops answering. The firewall row now follows from both: open
the traffic once the addresses and ports are agreed.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -824,23 +824,24 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="45" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Direcciones IP para exponer Kafka</t>
+          <t>Direcciones IP libres para exponer Kafka</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>La exposición se hace con un balanceador que toma direcciones de un rango del segmento de red del cluster. Se necesita una dirección por broker más una de entrada: 2 para desarrollo.</t>
+          <t>La exposición se hace con un balanceador que toma direcciones del segmento de red del cluster. Se necesita una por cada servidor de Kafka más una de entrada: 2 para desarrollo.
+Deben estar libres y reservadas para este uso: si otro equipo las ocupa, el servicio deja de responder.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Rango a definir con su equipo de redes</t>
+          <t>A definir con su equipo de redes</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
@@ -851,17 +852,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Puerto de conexión a Kafka</t>
+          <t>Puerto de conexión</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>El puerto por el que las aplicaciones se conectan al balanceador. Confirmar si el propuesto es válido según su normativa de red.</t>
+          <t>A definir por ustedes según su normativa. Se ocupan tantos puertos correlativos como direcciones: si se acuerda el 9094, en desarrollo se usarían el 9094 y el 9095.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>9094</t>
+          <t>A definir (propuesta: desde el 9094)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
@@ -877,7 +878,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Solo si están fuera: permitir el tránsito desde sus redes hacia esas direcciones y ese puerto. Indicar desde qué redes se originará.</t>
+          <t>Una vez definidas las direcciones y los puertos, habilitar el tránsito hacia ellos desde las redes donde se ejecutan las aplicaciones. Indicar cuáles son.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">

</xml_diff>

<commit_message>
fix: it is one port on every address, not consecutive ones
Checked against the Strimzi and Red Hat docs, and against the running cluster: the
operator creates one load-balancer Service per broker plus one for bootstrap, and
they all listen on the SAME port -- what differs is the IP. There is no 9095. The
cluster confirms it: two Services, both on 9094.

That matters because the bank sizes its firewall from this document, and the rule
has to open the port to ALL the addresses, not just the bootstrap one: a client
starts there but then talks to each broker directly. Opening only bootstrap is the
usual mistake -- it connects and then fails on send.

Also records that the port must be 9092 or above (443 is not accepted), that
retention is a guaranteed minimum since deletion happens in blocks, and that client
certificates expire and have to be renewed.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="75" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
@@ -672,7 +672,8 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan antes de eliminarse. Es una decisión de cumplimiento.</t>
+          <t>Cuánto tiempo se conservan antes de eliminarse. Es una decisión de cumplimiento.
+Es un mínimo garantizado: el borrado físico puede demorarse algo más, porque se hace por bloques y no evento a evento.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -835,7 +836,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>La exposición se hace con un balanceador que toma direcciones del segmento de red del cluster. Se necesita una por cada servidor de Kafka más una de entrada: 2 para desarrollo.
+          <t>Se necesita una dirección por cada servidor de Kafka más una de entrada: 2 en desarrollo (1 servidor) y 4 en los ambientes con 3 servidores.
 Deben estar libres y reservadas para este uso: si otro equipo las ocupa, el servicio deja de responder.</t>
         </is>
       </c>
@@ -857,17 +858,17 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>A definir por ustedes según su normativa. Se ocupan tantos puertos correlativos como direcciones: si se acuerda el 9094, en desarrollo se usarían el 9094 y el 9095.</t>
+          <t>A definir por ustedes: es UN solo puerto, el mismo en todas las direcciones. Debe ser el 9092 o superior; quedan reservados el 9404 y el 9999, y no se admiten puertos bajos como el 443.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>A definir (propuesta: desde el 9094)</t>
+          <t>A definir (propuesta: 9094)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="45" customHeight="1">
+    <row r="21" ht="105" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
@@ -878,7 +879,8 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Una vez definidas las direcciones y los puertos, habilitar el tránsito hacia ellos desde las redes donde se ejecutan las aplicaciones. Indicar cuáles son.</t>
+          <t>Permitir el tránsito hacia TODAS las direcciones por ese puerto, no solo hacia la de entrada: la aplicación empieza por ella, pero después conversa directamente con cada servidor.
+Abrir solo la de entrada es el error más habitual: conecta al principio y falla al enviar. Indicar desde qué redes se originará el tráfico.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -951,7 +953,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>19</v>
       </c>
@@ -962,7 +964,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta y cómo se les entrega.</t>
+          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta, cómo se les entrega y cómo se les renueva: los certificados caducan y hay que reemplazarlos antes de que expiren.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: ask for the thing instead of explaining around it
Every row described a topic and left the customer to infer what to send back.
Now each one names the deliverable -- 'two free IP addresses', 'the port we should
use', 'the list of fields holding personal data' -- and the explanation is whatever
still fits in one line after that.

The address count is spelled out per environment rather than left as a rule to
apply: development 2, the rest 4 each.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -539,18 +539,18 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Acceso al cluster de desarrollo</t>
+          <t>Usuario administrador en el cluster de desarrollo</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Credenciales de administrador para el equipo de implementación. Las condiciones técnicas del cluster las verificamos nosotros.</t>
+          <t>Para el equipo de implementación. Las condiciones técnicas del cluster las verificamos nosotros.</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -560,19 +560,18 @@
       </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="75" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Tres repositorios Git y acceso de administración</t>
+          <t>Tres repositorios Git vacíos, con permiso de administración</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Uno para el código del pipeline (Java), otro para el componente productor (.NET) y otro para la configuración de despliegue.
-La automatización la configuramos nosotros, pero su credencial debe emitirse desde su organización.</t>
+          <t>Uno para el código del pipeline (Java), otro para el componente productor (.NET) y otro para la configuración de despliegue. Incluir una credencial de su organización para la automatización.</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -599,7 +598,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Nombre del cluster de Kafka</t>
+          <t>El nombre que llevará el cluster de Kafka</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -620,7 +619,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Nombres de los cuatro tópicos</t>
+          <t>Los nombres de los cuatro tópicos</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -644,7 +643,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Nombres de los usuarios de Kafka</t>
+          <t>Los nombres de los tres usuarios de Kafka</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -661,19 +660,18 @@
       </c>
       <c r="E10" s="7" t="inlineStr"/>
     </row>
-    <row r="11" ht="75" customHeight="1">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Tiempo de retención de los eventos</t>
+          <t>Cuántas horas se conservan los eventos</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cuánto tiempo se conservan antes de eliminarse. Es una decisión de cumplimiento.
-Es un mínimo garantizado: el borrado físico puede demorarse algo más, porque se hace por bloques y no evento a evento.</t>
+          <t>Es una decisión de cumplimiento. El valor es un mínimo garantizado: el borrado puede demorarse algo más, porque se hace por bloques.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -690,12 +688,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Catálogo completo de datos personales</t>
+          <t>La lista completa de campos con datos personales</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Se enmascaran ÚNICAMENTE los campos que ustedes declaren: lo que no esté en la lista viaja sin enmascarar. Conviene revisarlo con el área de cumplimiento.</t>
+          <t>Se enmascaran ÚNICAMENTE los que ustedes declaren: lo que no esté en la lista viaja sin enmascarar. Conviene validarla con su área de cumplimiento.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -713,12 +711,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Volumen y tamaño de los eventos</t>
+          <t>Eventos por segundo y tamaño medio y máximo</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo, tamaño medio y máximo. De aquí sale el número de particiones, que después no se puede reducir.</t>
+          <t>De aquí sale el número de particiones, que después se puede aumentar pero no reducir.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -735,12 +733,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Destino final de los eventos enmascarados</t>
+          <t>El sistema destino de los eventos procesados</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>A dónde se entregan una vez procesados: sistema destino, punto de conexión y credenciales.</t>
+          <t>Con su punto de conexión y las credenciales de acceso.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -756,12 +754,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Aplicaciones que enviarán eventos</t>
+          <t>La lista de aplicaciones que enviarán eventos</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Cuáles integrarán el componente productor, para planificar la integración.</t>
+          <t>Las que integrarán el componente productor, para planificar la integración.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -777,12 +775,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Límites de consumo por aplicación</t>
+          <t>Confirmación de los límites de velocidad por aplicación</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Límite de velocidad por aplicación, para que un fallo en una no afecte a las demás.</t>
+          <t>Evitan que un fallo en una aplicación afecte a las demás.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -810,39 +808,38 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Dónde se ejecutan las aplicaciones</t>
+          <t>¿Sus aplicaciones se ejecutan dentro o fuera del cluster?</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Si están dentro del cluster no hay que abrir nada; si están fuera, hay que habilitar el tránsito hasta él.</t>
+          <t>Si están dentro, los puntos 13 a 15 no aplican.</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Se asume que están fuera del cluster</t>
+          <t>Fuera del cluster</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="90" customHeight="1">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Direcciones IP libres para exponer Kafka</t>
+          <t>2 direcciones IP libres del segmento del cluster</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Se necesita una dirección por cada servidor de Kafka más una de entrada: 2 en desarrollo (1 servidor) y 4 en los ambientes con 3 servidores.
-Deben estar libres y reservadas para este uso: si otro equipo las ocupa, el servicio deja de responder.</t>
+          <t>Una por cada servidor de Kafka más una de entrada. Por ambiente: desarrollo 2 · pruebas 4 · producción 4 · contingencia 4. Deben quedar reservadas para este uso.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>A definir con su equipo de redes</t>
+          <t>Para desarrollo: 2</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
@@ -853,34 +850,33 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Puerto de conexión</t>
+          <t>El puerto que debemos usar</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>A definir por ustedes: es UN solo puerto, el mismo en todas las direcciones. Debe ser el 9092 o superior; quedan reservados el 9404 y el 9999, y no se admiten puertos bajos como el 443.</t>
+          <t>Un único puerto, el mismo en todas las direcciones. Debe ser 9092 o superior (no se admiten 9404, 9999 ni puertos bajos como el 443).</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>A definir (propuesta: 9094)</t>
+          <t>Propuesta: 9094</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
-    <row r="21" ht="105" customHeight="1">
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red hacia Kafka</t>
+          <t>Reglas de firewall abiertas</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Permitir el tránsito hacia TODAS las direcciones por ese puerto, no solo hacia la de entrada: la aplicación empieza por ella, pero después conversa directamente con cada servidor.
-Abrir solo la de entrada es el error más habitual: conecta al principio y falla al enviar. Indicar desde qué redes se originará el tráfico.</t>
+          <t>Desde las redes de sus aplicaciones hacia LAS 2 DIRECCIONES, no solo hacia la de entrada. Indíquenos también desde qué redes se originará el tráfico.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -896,12 +892,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Habilitación de red desde el servidor Git</t>
+          <t>Regla de firewall desde su servidor Git hacia el cluster</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>El servidor Git avisa al cluster cuando alguien sube un cambio. Sin este permiso, la construcción no se dispara.</t>
+          <t>Para que avise cuando alguien sube un cambio y se lance la construcción.</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -917,12 +913,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Resolución de nombres</t>
+          <t>Confirmación de que sus servidores resuelven el dominio del cluster</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones se conectan por nombre. Confirmar que sus servidores resuelven el dominio del cluster.</t>
+          <t>Las aplicaciones se conectan por nombre, no por dirección IP.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -938,38 +934,38 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Confianza en el certificado del cluster</t>
+          <t>¿Quién emite el certificado del servidor: ustedes o nosotros?</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Las aplicaciones deben confiar en el certificado que presenta Kafka. Indicar si prefieren emitirlo con su autoridad corporativa.</t>
+          <t>Si lo emite su autoridad corporativa, necesitamos el certificado; si lo generamos nosotros, les entregamos el nuestro para que sus aplicaciones confíen en él.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Autoridad generada por la plataforma</t>
+          <t>Lo generamos nosotros</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr"/>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Identidad de cada aplicación productora</t>
+          <t>Número de identidades para sus aplicaciones</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Cada aplicación se autentica con su propio certificado. Cuántas identidades hacen falta, cómo se les entrega y cómo se les renueva: los certificados caducan y hay que reemplazarlos antes de que expiren.</t>
+          <t>Cada aplicación se autentica con su propio certificado, que emitimos nosotros. Indíquenos cuántas hacen falta y a quién se las entregamos. Caducan y hay que renovarlas.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Una identidad compartida por ambiente</t>
+          <t>Una identidad por ambiente</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr"/>
@@ -985,18 +981,18 @@
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="5" t="n">
         <v>20</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Repositorio interno de paquetes .NET</t>
+          <t>Un repositorio interno de paquetes .NET</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Sus equipos incorporan el componente como dependencia: hace falta un repositorio interno donde publicarlo.</t>
+          <t>Con permiso de publicación para nosotros y de lectura para sus equipos: es de donde sus aplicaciones descargarán el componente.</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1012,12 +1008,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Versión de .NET de las aplicaciones</t>
+          <t>La versión de .NET de sus aplicaciones</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>El componente está construido sobre .NET 10. Confirmar la versión de las aplicaciones que lo integrarán.</t>
+          <t>El componente está construido sobre .NET 10 y requiere esa versión o superior.</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1044,12 +1040,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Llave de cifrado en Azure Key Vault</t>
+          <t>El Key Vault a utilizar y el nombre del secreto</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Se deposita en el Key Vault y desde ahí se sincroniza al cluster. Confirmar cuál usar y el nombre del secreto.</t>
+          <t>Ahí depositan la llave de cifrado; desde ahí se sincroniza sola al cluster.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1065,12 +1061,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Acceso de OpenShift al Key Vault</t>
+          <t>Una identidad de Azure con lectura sobre ese Key Vault</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Una identidad de Azure con permiso de lectura sobre el Key Vault.</t>
+          <t>Es con la que el cluster obtiene la llave.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1086,12 +1082,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Política de rotación de la llave</t>
+          <t>Cada cuánto debe rotarse la llave de cifrado</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse. La rotación no pierde los eventos ya publicados.</t>
+          <t>La rotación no pierde los eventos ya publicados.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -1107,12 +1103,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Entrega de credenciales a aplicaciones externas</t>
+          <t>Cómo entregamos las credenciales a sus aplicaciones</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Solo si hay aplicaciones fuera del cluster: cómo se les hace llegar su certificado y la llave.</t>
+          <t>Solo si se ejecutan fuera del cluster: necesitan su certificado y la llave de cifrado en su servidor.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -1128,12 +1124,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Custodia de la llave de firma</t>
+          <t>Quién custodia la llave con la que se firman las imágenes</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Las imágenes se firman para verificar su origen. Definir quién custodia la llave.</t>
+          <t>La generamos nosotros; la firma permite verificar el origen de cada imagen.</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: say why Kafka needs an address per broker
The per-environment counts read as arbitrary without the reason behind them. A
client connects to the bootstrap address, gets back the list of servers, and from
there talks to each one directly -- so every broker needs its own reachable
address. Development runs one broker, the other environments run three so the
service survives losing one.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="45" customHeight="1">
+    <row r="19" ht="150" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
@@ -834,12 +834,17 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Una por cada servidor de Kafka más una de entrada. Por ambiente: desarrollo 2 · pruebas 4 · producción 4 · contingencia 4. Deben quedar reservadas para este uso.</t>
+          <t>Kafka no funciona con una sola dirección: la aplicación se conecta a la de entrada, que le devuelve la lista de servidores, y a partir de ahí habla directamente con cada uno. Por eso cada servidor necesita su propia dirección alcanzable.
+Desarrollo tiene 1 servidor (1 + entrada = 2 direcciones). Los demás ambientes tienen 3, para que el servicio siga funcionando si cae uno (3 + entrada = 4 direcciones).
+Deben quedar reservadas para este uso.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Para desarrollo: 2</t>
+          <t>Desarrollo: 2
+Pruebas: 4
+Producción: 4
+Contingencia: 4</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: state that MetalLB is required on the customer's own hardware
The workload ApplicationSets left MetalLB commented out with a note pointing at a
use_metallb variable that does not exist anywhere. It stays commented because this
cluster runs in a cloud that provisions load balancers itself -- but the customer
installs on their own servers, where without MetalLB every LoadBalancer Service sits
in Pending and Kafka is never reachable. The comment now says that.

The address row asks for real IPs from their segment, contiguous and reserved, plus
the netmask and gateway MetalLB needs to advertise them.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -823,20 +823,20 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
     </row>
-    <row r="19" ht="150" customHeight="1">
+    <row r="19" ht="195" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>2 direcciones IP libres del segmento del cluster</t>
+          <t>2 direcciones de red para exponer Kafka</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Kafka no funciona con una sola dirección: la aplicación se conecta a la de entrada, que le devuelve la lista de servidores, y a partir de ahí habla directamente con cada uno. Por eso cada servidor necesita su propia dirección alcanzable.
-Desarrollo tiene 1 servidor (1 + entrada = 2 direcciones). Los demás ambientes tienen 3, para que el servicio siga funcionando si cae uno (3 + entrada = 4 direcciones).
-Deben quedar reservadas para este uso.</t>
+          <t>Kafka no funciona con una sola: la aplicación se conecta a la de entrada, que le devuelve la lista de servidores, y a partir de ahí habla directamente con cada uno. Cada servidor necesita la suya.
+Desarrollo tiene 1 servidor (1 + entrada = 2). Los demás ambientes tienen 3, para que el servicio siga funcionando si cae uno (3 + entrada = 4).
+Son IPs de su segmento de red, contiguas y reservadas para este uso: si otro equipo las ocupa, el servicio deja de responder. Indíquenos también la máscara y la puerta de enlace del segmento.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: call them brokers, which is what they are
The address row said 'servers'. Kafka calls them brokers, it is what the pods are
named, and it is the word the customer will meet in every log and dashboard --
introduced once so a network engineer can still follow the count.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -834,8 +834,8 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Kafka no funciona con una sola: la aplicación se conecta a la de entrada, que le devuelve la lista de servidores, y a partir de ahí habla directamente con cada uno. Cada servidor necesita la suya.
-Desarrollo tiene 1 servidor (1 + entrada = 2). Los demás ambientes tienen 3, para que el servicio siga funcionando si cae uno (3 + entrada = 4).
+          <t>Kafka no funciona con una sola: la aplicación se conecta a la de entrada, que le devuelve la lista de nodos (en Kafka se llaman BROKERS), y a partir de ahí habla directamente con cada uno. Cada broker necesita la suya.
+Desarrollo tiene 1 broker (1 + entrada = 2). Los demás ambientes tienen 3, para que el servicio siga funcionando si cae uno (3 + entrada = 4).
 Son IPs de su segmento de red, contiguas y reservadas para este uso: si otro equipo las ocupa, el servicio deja de responder. Indíquenos también la máscara y la puerta de enlace del segmento.</t>
         </is>
       </c>
@@ -939,7 +939,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>¿Quién emite el certificado del servidor: ustedes o nosotros?</t>
+          <t>¿Quién emite el certificado de Kafka: ustedes o nosotros?</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: name each ask with the term it actually has
Vague titles made the reader guess: 'the port we should use' is a listener port,
'reserved addresses' are the ones MetalLB hands out, 'identities' are mTLS client
certificates. Each row now carries the real term -- cluster-admin, KafkaUser, CA,
NuGet, Key Vault -- so the right team recognises its own work at a glance, with the
plain-language explanation still underneath.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Usuario administrador en el cluster de desarrollo</t>
+          <t>Usuario con rol cluster-admin en el cluster de desarrollo</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Tres repositorios Git vacíos, con permiso de administración</t>
+          <t>Tres repositorios Git vacíos, con rol de administrador</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>El nombre que llevará el cluster de Kafka</t>
+          <t>Nombre del cluster de Kafka</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Los nombres de los cuatro tópicos</t>
+          <t>Nombres de los cuatro tópicos (topics)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Los nombres de los tres usuarios de Kafka</t>
+          <t>Nombres de los tres usuarios de Kafka (KafkaUser)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Cuántas horas se conservan los eventos</t>
+          <t>Retención de los eventos, en horas</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>La lista completa de campos con datos personales</t>
+          <t>Campos con datos personales que deben enmascararse</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Eventos por segundo y tamaño medio y máximo</t>
+          <t>Volumen: eventos por segundo y tamaño medio y máximo</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>El sistema destino de los eventos procesados</t>
+          <t>Sistema destino de los eventos ya procesados</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>La lista de aplicaciones que enviarán eventos</t>
+          <t>Aplicaciones que actuarán como productoras de eventos</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Confirmación de los límites de velocidad por aplicación</t>
+          <t>Cuotas de throughput por aplicación</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>¿Sus aplicaciones se ejecutan dentro o fuera del cluster?</t>
+          <t>¿Sus aplicaciones corren dentro o fuera del cluster?</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>2 direcciones de red para exponer Kafka</t>
+          <t>2 direcciones IP para los balanceadores de Kafka (MetalLB)</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>El puerto que debemos usar</t>
+          <t>Puerto TCP del listener externo de Kafka</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Reglas de firewall abiertas</t>
+          <t>Reglas de firewall hacia Kafka</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Confirmación de que sus servidores resuelven el dominio del cluster</t>
+          <t>Resolución DNS del dominio del cluster</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>¿Quién emite el certificado de Kafka: ustedes o nosotros?</t>
+          <t>Autoridad certificadora (CA) del certificado de Kafka</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Número de identidades para sus aplicaciones</t>
+          <t>Número de certificados de cliente (mTLS) para sus aplicaciones</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Un repositorio interno de paquetes .NET</t>
+          <t>Repositorio interno de paquetes NuGet</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>La versión de .NET de sus aplicaciones</t>
+          <t>Versión de .NET de sus aplicaciones</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>El Key Vault a utilizar y el nombre del secreto</t>
+          <t>Azure Key Vault y nombre del secreto de la llave</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Una identidad de Azure con lectura sobre ese Key Vault</t>
+          <t>Identidad de Azure con permiso de lectura sobre el Key Vault</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Cada cuánto debe rotarse la llave de cifrado</t>
+          <t>Periodicidad de rotación de la llave de cifrado</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Cómo entregamos las credenciales a sus aplicaciones</t>
+          <t>Mecanismo de entrega de credenciales a sus aplicaciones</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Quién custodia la llave con la que se firman las imágenes</t>
+          <t>Custodia de la llave de firma de imágenes</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: trim the header note to one sentence
It listed what we verify ourselves and restated the column meanings -- detail the
reader does not need before starting. Two lines: who installs, and what to do with
the sheet.
</commit_message>
<xml_diff>
--- a/docs/prerrequisitos-kafka-dev.xlsx
+++ b/docs/prerrequisitos-kafka-dev.xlsx
@@ -494,10 +494,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="34" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>La instalación y configuración las realiza el equipo de implementación, que también verifica las condiciones técnicas del cluster (almacenamiento, capacidad, conectividad y versiones). Este documento recoge únicamente lo que necesitamos de su parte: accesos, definiciones de negocio y decisiones de gobierno. Puede completar la última columna y devolvernos el fichero; si algún punto no se define, se aplicará el valor indicado en la columna anterior.</t>
+          <t>La instalación la realiza el equipo de implementación. Aquí recogemos lo que necesitamos de su parte: complete la última columna y devuélvanos el archivo. Si un punto no se define, se aplicará el valor de la columna anterior.</t>
         </is>
       </c>
     </row>

</xml_diff>